<commit_message>
vault backup: 2026-08-15 00:52:44
</commit_message>
<xml_diff>
--- a/00_SBG/07_ライブラリ/外部資料/sample_Ver.0.25.xlsx
+++ b/00_SBG/07_ライブラリ/外部資料/sample_Ver.0.25.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\payla\Documents\GitHub\SBG_Obsidian\00_SBG\07_ライブラリ\外部資料\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\playn\Documents\Github\SBG_Obsidian\00_SBG\07_ライブラリ\外部資料\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C08DF11-C73D-451A-B7CB-7D4675225F0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D829C7DF-4426-4874-B6A6-95087BEFDDD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-10910" windowWidth="19420" windowHeight="11020" firstSheet="9" activeTab="13" xr2:uid="{1AFB224D-C5F6-4405-A264-ECF4615FFB57}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{1AFB224D-C5F6-4405-A264-ECF4615FFB57}"/>
   </bookViews>
   <sheets>
     <sheet name="Character" sheetId="1" r:id="rId1"/>
@@ -1844,26 +1844,26 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55B8B1C1-796A-41F2-87F3-C69DB116ED24}">
   <dimension ref="A1:Q19"/>
-  <sheetFormatPr defaultRowHeight="17.649999999999999" x14ac:dyDescent="0.7"/>
+  <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="12.375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.3984375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.5" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="7.125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="6.6875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7.09765625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.3984375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.3984375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="6.69921875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="16" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.8984375" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="9" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="13.875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.8984375" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="27.5" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="14.5" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="18.125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="18.09765625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.7">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1916,7 +1916,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.7">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>17</v>
       </c>
@@ -1969,7 +1969,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.7">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>19</v>
       </c>
@@ -2022,7 +2022,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.7">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>155</v>
       </c>
@@ -2075,7 +2075,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.7">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>156</v>
       </c>
@@ -2128,7 +2128,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.7">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>157</v>
       </c>
@@ -2181,7 +2181,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.7">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>177</v>
       </c>
@@ -2234,7 +2234,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.7">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>178</v>
       </c>
@@ -2287,7 +2287,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.7">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>89</v>
       </c>
@@ -2340,7 +2340,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.7">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>90</v>
       </c>
@@ -2393,7 +2393,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.7">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>123</v>
       </c>
@@ -2446,7 +2446,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.7">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>124</v>
       </c>
@@ -2499,7 +2499,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.7">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
         <v>162</v>
       </c>
@@ -2552,7 +2552,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.7">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
         <v>217</v>
       </c>
@@ -2605,7 +2605,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="19" spans="3:3" x14ac:dyDescent="0.7">
+    <row r="19" spans="3:3" x14ac:dyDescent="0.45">
       <c r="C19" s="2"/>
     </row>
   </sheetData>
@@ -2620,14 +2620,14 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4756A621-9C73-46F6-BCC6-EFA4C1E375C5}">
   <dimension ref="A1:C10"/>
-  <sheetFormatPr defaultRowHeight="17.649999999999999" x14ac:dyDescent="0.7"/>
+  <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="13.625" customWidth="1"/>
-    <col min="2" max="2" width="13.6875" customWidth="1"/>
-    <col min="3" max="3" width="7.625" customWidth="1"/>
+    <col min="1" max="1" width="13.59765625" customWidth="1"/>
+    <col min="2" max="2" width="13.69921875" customWidth="1"/>
+    <col min="3" max="3" width="7.59765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.7">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>46</v>
       </c>
@@ -2638,7 +2638,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.7">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>27</v>
       </c>
@@ -2649,7 +2649,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.7">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>27</v>
       </c>
@@ -2660,7 +2660,7 @@
         <v>1.2</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.7">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>27</v>
       </c>
@@ -2671,7 +2671,7 @@
         <v>0.8</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.7">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>28</v>
       </c>
@@ -2682,7 +2682,7 @@
         <v>0.8</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.7">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>28</v>
       </c>
@@ -2693,7 +2693,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.7">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>28</v>
       </c>
@@ -2704,7 +2704,7 @@
         <v>1.2</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.7">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>29</v>
       </c>
@@ -2715,7 +2715,7 @@
         <v>1.2</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.7">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>29</v>
       </c>
@@ -2726,7 +2726,7 @@
         <v>0.8</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.7">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>29</v>
       </c>
@@ -2749,14 +2749,14 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45C69C40-D8C8-4D84-9DB2-2ED24622B6ED}">
   <dimension ref="A1:D6"/>
-  <sheetFormatPr defaultRowHeight="17.649999999999999" x14ac:dyDescent="0.7"/>
+  <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="9.875" customWidth="1"/>
-    <col min="2" max="2" width="11.625" customWidth="1"/>
-    <col min="3" max="3" width="6.875" customWidth="1"/>
+    <col min="1" max="1" width="9.8984375" customWidth="1"/>
+    <col min="2" max="2" width="11.59765625" customWidth="1"/>
+    <col min="3" max="3" width="6.8984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.7">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -2767,7 +2767,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.7">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A2">
         <v>1</v>
       </c>
@@ -2778,7 +2778,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.7">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A3">
         <v>2</v>
       </c>
@@ -2789,10 +2789,10 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.7">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A4" s="2"/>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.7">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.45">
       <c r="D6" s="2"/>
     </row>
   </sheetData>
@@ -2807,14 +2807,14 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D85222A2-312A-4ED7-934F-358F77FC3BC8}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="17.649999999999999" x14ac:dyDescent="0.7"/>
+  <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="18.875" customWidth="1"/>
-    <col min="2" max="2" width="11.6875" customWidth="1"/>
-    <col min="3" max="3" width="14.375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.8984375" customWidth="1"/>
+    <col min="2" max="2" width="11.69921875" customWidth="1"/>
+    <col min="3" max="3" width="14.3984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.7">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>52</v>
       </c>
@@ -2825,7 +2825,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.7">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>97</v>
       </c>
@@ -2836,7 +2836,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.7">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>96</v>
       </c>
@@ -2847,7 +2847,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.7">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>168</v>
       </c>
@@ -2858,7 +2858,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.7">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>169</v>
       </c>
@@ -2869,7 +2869,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.7">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>170</v>
       </c>
@@ -2880,7 +2880,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.7">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>215</v>
       </c>
@@ -2903,13 +2903,13 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0CEAA3CD-9992-44D9-9B4B-D14DBC9A2B99}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultRowHeight="17.649999999999999" x14ac:dyDescent="0.7"/>
+  <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="11.625" customWidth="1"/>
+    <col min="1" max="1" width="11.59765625" customWidth="1"/>
     <col min="2" max="2" width="16.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.7">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>41</v>
       </c>
@@ -2917,7 +2917,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.7">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>121</v>
       </c>
@@ -2925,7 +2925,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.7">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>122</v>
       </c>
@@ -2945,35 +2945,35 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A8E5DC47-9D66-441C-BA5C-D7967849AB01}">
   <dimension ref="A1:Y49"/>
-  <sheetFormatPr defaultRowHeight="17.649999999999999" x14ac:dyDescent="0.7"/>
+  <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="24.1875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="24.19921875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9.5" customWidth="1"/>
-    <col min="3" max="3" width="9.875" customWidth="1"/>
-    <col min="4" max="4" width="9.625" customWidth="1"/>
+    <col min="3" max="3" width="9.8984375" customWidth="1"/>
+    <col min="4" max="4" width="9.59765625" customWidth="1"/>
     <col min="5" max="5" width="15.5" customWidth="1"/>
     <col min="6" max="6" width="9" customWidth="1"/>
     <col min="7" max="7" width="10.5" customWidth="1"/>
     <col min="8" max="8" width="17.5" customWidth="1"/>
     <col min="9" max="9" width="14.5" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="20.875" customWidth="1"/>
-    <col min="11" max="11" width="17.1875" customWidth="1"/>
-    <col min="12" max="12" width="17.375" customWidth="1"/>
-    <col min="13" max="13" width="16.875" customWidth="1"/>
-    <col min="14" max="14" width="18.1875" customWidth="1"/>
-    <col min="15" max="15" width="25.375" customWidth="1"/>
-    <col min="16" max="17" width="24.6875" customWidth="1"/>
-    <col min="18" max="18" width="10.125" customWidth="1"/>
-    <col min="19" max="19" width="17.625" customWidth="1"/>
-    <col min="20" max="20" width="12.6875" customWidth="1"/>
-    <col min="21" max="21" width="12.125" customWidth="1"/>
-    <col min="22" max="22" width="13.6875" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="15.6875" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="19.375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="20.8984375" customWidth="1"/>
+    <col min="11" max="11" width="17.19921875" customWidth="1"/>
+    <col min="12" max="12" width="17.3984375" customWidth="1"/>
+    <col min="13" max="13" width="16.8984375" customWidth="1"/>
+    <col min="14" max="14" width="18.19921875" customWidth="1"/>
+    <col min="15" max="15" width="25.3984375" customWidth="1"/>
+    <col min="16" max="17" width="24.69921875" customWidth="1"/>
+    <col min="18" max="18" width="10.09765625" customWidth="1"/>
+    <col min="19" max="19" width="17.59765625" customWidth="1"/>
+    <col min="20" max="20" width="12.69921875" customWidth="1"/>
+    <col min="21" max="21" width="12.09765625" customWidth="1"/>
+    <col min="22" max="22" width="13.69921875" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="15.69921875" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="19.3984375" bestFit="1" customWidth="1"/>
     <col min="25" max="25" width="12.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" x14ac:dyDescent="0.7">
+    <row r="1" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -3050,7 +3050,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="2" spans="1:25" x14ac:dyDescent="0.7">
+    <row r="2" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>115</v>
       </c>
@@ -3127,7 +3127,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:25" x14ac:dyDescent="0.7">
+    <row r="3" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>114</v>
       </c>
@@ -3204,7 +3204,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:25" x14ac:dyDescent="0.7">
+    <row r="4" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>207</v>
       </c>
@@ -3281,7 +3281,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:25" x14ac:dyDescent="0.7">
+    <row r="5" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>208</v>
       </c>
@@ -3358,7 +3358,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:25" x14ac:dyDescent="0.7">
+    <row r="6" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>209</v>
       </c>
@@ -3435,7 +3435,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:25" x14ac:dyDescent="0.7">
+    <row r="7" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>116</v>
       </c>
@@ -3509,7 +3509,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:25" x14ac:dyDescent="0.7">
+    <row r="8" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>192</v>
       </c>
@@ -3583,7 +3583,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:25" x14ac:dyDescent="0.7">
+    <row r="9" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>117</v>
       </c>
@@ -3657,7 +3657,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="10" spans="1:25" x14ac:dyDescent="0.7">
+    <row r="10" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>143</v>
       </c>
@@ -3731,7 +3731,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:25" x14ac:dyDescent="0.7">
+    <row r="11" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>194</v>
       </c>
@@ -3805,7 +3805,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:25" x14ac:dyDescent="0.7">
+    <row r="12" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>144</v>
       </c>
@@ -3879,7 +3879,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="13" spans="1:25" x14ac:dyDescent="0.7">
+    <row r="13" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
         <v>193</v>
       </c>
@@ -3953,7 +3953,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="1:25" x14ac:dyDescent="0.7">
+    <row r="14" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
         <v>195</v>
       </c>
@@ -4027,7 +4027,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:25" x14ac:dyDescent="0.7">
+    <row r="15" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
         <v>219</v>
       </c>
@@ -4101,7 +4101,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="16" spans="1:25" x14ac:dyDescent="0.7">
+    <row r="16" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
         <v>71</v>
       </c>
@@ -4175,7 +4175,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:25" x14ac:dyDescent="0.7">
+    <row r="17" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
         <v>72</v>
       </c>
@@ -4249,7 +4249,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:25" x14ac:dyDescent="0.7">
+    <row r="18" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
         <v>121</v>
       </c>
@@ -4323,7 +4323,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:25" x14ac:dyDescent="0.7">
+    <row r="19" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
         <v>122</v>
       </c>
@@ -4397,7 +4397,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="20" spans="1:25" x14ac:dyDescent="0.7">
+    <row r="20" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
         <v>85</v>
       </c>
@@ -4471,7 +4471,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:25" x14ac:dyDescent="0.7">
+    <row r="21" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
         <v>92</v>
       </c>
@@ -4545,7 +4545,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:25" x14ac:dyDescent="0.7">
+    <row r="22" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
         <v>95</v>
       </c>
@@ -4619,7 +4619,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:25" x14ac:dyDescent="0.7">
+    <row r="23" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
         <v>102</v>
       </c>
@@ -4693,7 +4693,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="24" spans="1:25" x14ac:dyDescent="0.7">
+    <row r="24" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
         <v>107</v>
       </c>
@@ -4767,7 +4767,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:25" x14ac:dyDescent="0.7">
+    <row r="25" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
         <v>103</v>
       </c>
@@ -4841,7 +4841,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="26" spans="1:25" x14ac:dyDescent="0.7">
+    <row r="26" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
         <v>108</v>
       </c>
@@ -4915,7 +4915,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:25" x14ac:dyDescent="0.7">
+    <row r="27" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
         <v>104</v>
       </c>
@@ -4989,7 +4989,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:25" x14ac:dyDescent="0.7">
+    <row r="28" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
         <v>146</v>
       </c>
@@ -5063,7 +5063,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:25" x14ac:dyDescent="0.7">
+    <row r="29" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
         <v>147</v>
       </c>
@@ -5140,7 +5140,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="30" spans="1:25" x14ac:dyDescent="0.7">
+    <row r="30" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A30" t="s">
         <v>149</v>
       </c>
@@ -5214,7 +5214,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:25" x14ac:dyDescent="0.7">
+    <row r="31" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A31" t="s">
         <v>150</v>
       </c>
@@ -5291,7 +5291,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="32" spans="1:25" x14ac:dyDescent="0.7">
+    <row r="32" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A32" t="s">
         <v>152</v>
       </c>
@@ -5365,7 +5365,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:25" x14ac:dyDescent="0.7">
+    <row r="33" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A33" t="s">
         <v>153</v>
       </c>
@@ -5439,7 +5439,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="34" spans="1:25" x14ac:dyDescent="0.7">
+    <row r="34" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A34" t="s">
         <v>197</v>
       </c>
@@ -5513,7 +5513,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:25" x14ac:dyDescent="0.7">
+    <row r="35" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A35" t="s">
         <v>198</v>
       </c>
@@ -5587,7 +5587,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="36" spans="1:25" x14ac:dyDescent="0.7">
+    <row r="36" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A36" t="s">
         <v>199</v>
       </c>
@@ -5661,7 +5661,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:25" x14ac:dyDescent="0.7">
+    <row r="37" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A37" t="s">
         <v>200</v>
       </c>
@@ -5735,7 +5735,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:25" x14ac:dyDescent="0.7">
+    <row r="38" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A38" t="s">
         <v>201</v>
       </c>
@@ -5809,7 +5809,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:25" x14ac:dyDescent="0.7">
+    <row r="39" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A39" t="s">
         <v>202</v>
       </c>
@@ -5883,7 +5883,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="40" spans="1:25" x14ac:dyDescent="0.7">
+    <row r="40" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A40" t="s">
         <v>203</v>
       </c>
@@ -5957,7 +5957,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:25" x14ac:dyDescent="0.7">
+    <row r="41" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A41" t="s">
         <v>204</v>
       </c>
@@ -6031,7 +6031,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:25" x14ac:dyDescent="0.7">
+    <row r="42" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A42" t="s">
         <v>205</v>
       </c>
@@ -6108,7 +6108,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:25" x14ac:dyDescent="0.7">
+    <row r="43" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A43" t="s">
         <v>206</v>
       </c>
@@ -6182,7 +6182,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="44" spans="1:25" x14ac:dyDescent="0.7">
+    <row r="44" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A44" t="s">
         <v>110</v>
       </c>
@@ -6256,7 +6256,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="1:25" x14ac:dyDescent="0.7">
+    <row r="45" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A45" t="s">
         <v>105</v>
       </c>
@@ -6330,7 +6330,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="46" spans="1:25" x14ac:dyDescent="0.7">
+    <row r="46" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A46" t="s">
         <v>109</v>
       </c>
@@ -6404,7 +6404,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="47" spans="1:25" x14ac:dyDescent="0.7">
+    <row r="47" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A47" t="s">
         <v>106</v>
       </c>
@@ -6478,7 +6478,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="48" spans="1:25" x14ac:dyDescent="0.7">
+    <row r="48" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A48" t="s">
         <v>216</v>
       </c>
@@ -6555,7 +6555,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="2:25" x14ac:dyDescent="0.7">
+    <row r="49" spans="2:25" x14ac:dyDescent="0.45">
       <c r="B49">
         <v>0</v>
       </c>
@@ -6638,14 +6638,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ECE8E980-9D75-4087-B4F8-F29B93410A36}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="17.649999999999999" x14ac:dyDescent="0.7"/>
+  <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="10.5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="31.5625" customWidth="1"/>
+    <col min="2" max="2" width="31.59765625" customWidth="1"/>
     <col min="3" max="3" width="14.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.7">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -6656,7 +6656,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.7">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>93</v>
       </c>
@@ -6667,7 +6667,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.7">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>94</v>
       </c>
@@ -6678,7 +6678,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.7">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>84</v>
       </c>
@@ -6701,17 +6701,17 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{646309C0-1AC1-40CF-851B-3BE46F905216}">
   <dimension ref="A1:F11"/>
-  <sheetFormatPr defaultRowHeight="17.649999999999999" x14ac:dyDescent="0.7"/>
+  <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="15.375" customWidth="1"/>
-    <col min="2" max="2" width="10.625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.3984375" customWidth="1"/>
+    <col min="2" max="2" width="10.59765625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.59765625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="18" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.7">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -6731,7 +6731,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.7">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>131</v>
       </c>
@@ -6751,7 +6751,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.7">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>91</v>
       </c>
@@ -6771,7 +6771,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.7">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>159</v>
       </c>
@@ -6791,7 +6791,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.7">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>158</v>
       </c>
@@ -6811,7 +6811,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.7">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>160</v>
       </c>
@@ -6831,7 +6831,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.7">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>164</v>
       </c>
@@ -6851,7 +6851,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.7">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>163</v>
       </c>
@@ -6871,7 +6871,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.7">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>134</v>
       </c>
@@ -6891,7 +6891,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.7">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>135</v>
       </c>
@@ -6911,7 +6911,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.7">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>133</v>
       </c>
@@ -6943,16 +6943,16 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3094CBAF-F9CC-42AA-93E3-0E10EDB827F2}">
   <dimension ref="A1:E101"/>
-  <sheetFormatPr defaultRowHeight="17.649999999999999" x14ac:dyDescent="0.7"/>
+  <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
-    <col min="2" max="2" width="11.875" customWidth="1"/>
-    <col min="3" max="3" width="12.1875" customWidth="1"/>
-    <col min="4" max="4" width="12.625" customWidth="1"/>
+    <col min="2" max="2" width="11.8984375" customWidth="1"/>
+    <col min="3" max="3" width="12.19921875" customWidth="1"/>
+    <col min="4" max="4" width="12.59765625" customWidth="1"/>
     <col min="5" max="5" width="23.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>9</v>
       </c>
@@ -6969,7 +6969,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A2">
         <v>1</v>
       </c>
@@ -6986,7 +6986,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A3">
         <v>2</v>
       </c>
@@ -7003,7 +7003,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A4">
         <v>3</v>
       </c>
@@ -7020,7 +7020,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A5">
         <v>4</v>
       </c>
@@ -7037,7 +7037,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A6">
         <v>5</v>
       </c>
@@ -7054,7 +7054,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A7">
         <v>6</v>
       </c>
@@ -7071,7 +7071,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A8">
         <v>7</v>
       </c>
@@ -7088,7 +7088,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A9">
         <v>8</v>
       </c>
@@ -7105,7 +7105,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A10">
         <v>9</v>
       </c>
@@ -7122,7 +7122,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A11">
         <v>10</v>
       </c>
@@ -7139,7 +7139,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A12">
         <v>11</v>
       </c>
@@ -7156,7 +7156,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A13">
         <v>12</v>
       </c>
@@ -7173,7 +7173,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A14">
         <v>13</v>
       </c>
@@ -7190,7 +7190,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A15">
         <v>14</v>
       </c>
@@ -7207,7 +7207,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A16">
         <v>15</v>
       </c>
@@ -7224,7 +7224,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A17">
         <v>16</v>
       </c>
@@ -7241,7 +7241,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A18">
         <v>17</v>
       </c>
@@ -7258,7 +7258,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A19">
         <v>18</v>
       </c>
@@ -7275,7 +7275,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A20">
         <v>19</v>
       </c>
@@ -7292,7 +7292,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A21">
         <v>20</v>
       </c>
@@ -7309,7 +7309,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A22">
         <v>21</v>
       </c>
@@ -7326,7 +7326,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A23">
         <v>22</v>
       </c>
@@ -7343,7 +7343,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A24">
         <v>23</v>
       </c>
@@ -7360,7 +7360,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A25">
         <v>24</v>
       </c>
@@ -7377,7 +7377,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A26">
         <v>25</v>
       </c>
@@ -7394,7 +7394,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A27">
         <v>26</v>
       </c>
@@ -7411,7 +7411,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A28">
         <v>27</v>
       </c>
@@ -7428,7 +7428,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A29">
         <v>28</v>
       </c>
@@ -7445,7 +7445,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A30">
         <v>29</v>
       </c>
@@ -7462,7 +7462,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A31">
         <v>30</v>
       </c>
@@ -7479,7 +7479,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A32">
         <v>31</v>
       </c>
@@ -7496,7 +7496,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A33">
         <v>32</v>
       </c>
@@ -7513,7 +7513,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A34">
         <v>33</v>
       </c>
@@ -7530,7 +7530,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A35">
         <v>34</v>
       </c>
@@ -7547,7 +7547,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A36">
         <v>35</v>
       </c>
@@ -7564,7 +7564,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A37">
         <v>36</v>
       </c>
@@ -7581,7 +7581,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A38">
         <v>37</v>
       </c>
@@ -7598,7 +7598,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A39">
         <v>38</v>
       </c>
@@ -7615,7 +7615,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A40">
         <v>39</v>
       </c>
@@ -7632,7 +7632,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A41">
         <v>40</v>
       </c>
@@ -7649,7 +7649,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A42">
         <v>41</v>
       </c>
@@ -7666,7 +7666,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A43">
         <v>42</v>
       </c>
@@ -7683,7 +7683,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A44">
         <v>43</v>
       </c>
@@ -7700,7 +7700,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A45">
         <v>44</v>
       </c>
@@ -7717,7 +7717,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A46">
         <v>45</v>
       </c>
@@ -7734,7 +7734,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A47">
         <v>46</v>
       </c>
@@ -7751,7 +7751,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A48">
         <v>47</v>
       </c>
@@ -7768,7 +7768,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A49">
         <v>48</v>
       </c>
@@ -7785,7 +7785,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A50">
         <v>49</v>
       </c>
@@ -7802,7 +7802,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A51">
         <v>50</v>
       </c>
@@ -7819,7 +7819,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A52">
         <v>51</v>
       </c>
@@ -7836,7 +7836,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A53">
         <v>52</v>
       </c>
@@ -7853,7 +7853,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A54">
         <v>53</v>
       </c>
@@ -7870,7 +7870,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A55">
         <v>54</v>
       </c>
@@ -7887,7 +7887,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A56">
         <v>55</v>
       </c>
@@ -7904,7 +7904,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A57">
         <v>56</v>
       </c>
@@ -7921,7 +7921,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A58">
         <v>57</v>
       </c>
@@ -7938,7 +7938,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A59">
         <v>58</v>
       </c>
@@ -7955,7 +7955,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A60">
         <v>59</v>
       </c>
@@ -7972,7 +7972,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A61">
         <v>60</v>
       </c>
@@ -7989,7 +7989,7 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A62">
         <v>61</v>
       </c>
@@ -8006,7 +8006,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A63">
         <v>62</v>
       </c>
@@ -8023,7 +8023,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A64">
         <v>63</v>
       </c>
@@ -8040,7 +8040,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A65">
         <v>64</v>
       </c>
@@ -8057,7 +8057,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A66">
         <v>65</v>
       </c>
@@ -8074,7 +8074,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A67">
         <v>66</v>
       </c>
@@ -8091,7 +8091,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A68">
         <v>67</v>
       </c>
@@ -8108,7 +8108,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A69">
         <v>68</v>
       </c>
@@ -8125,7 +8125,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A70">
         <v>69</v>
       </c>
@@ -8142,7 +8142,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A71">
         <v>70</v>
       </c>
@@ -8159,7 +8159,7 @@
         <v>0.35</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A72">
         <v>71</v>
       </c>
@@ -8176,7 +8176,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A73">
         <v>72</v>
       </c>
@@ -8193,7 +8193,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A74">
         <v>73</v>
       </c>
@@ -8210,7 +8210,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A75">
         <v>74</v>
       </c>
@@ -8227,7 +8227,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A76">
         <v>75</v>
       </c>
@@ -8244,7 +8244,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A77">
         <v>76</v>
       </c>
@@ -8261,7 +8261,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A78">
         <v>77</v>
       </c>
@@ -8278,7 +8278,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A79">
         <v>78</v>
       </c>
@@ -8295,7 +8295,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A80">
         <v>79</v>
       </c>
@@ -8312,7 +8312,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A81">
         <v>80</v>
       </c>
@@ -8329,7 +8329,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A82">
         <v>81</v>
       </c>
@@ -8346,7 +8346,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A83">
         <v>82</v>
       </c>
@@ -8363,7 +8363,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A84">
         <v>83</v>
       </c>
@@ -8380,7 +8380,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A85">
         <v>84</v>
       </c>
@@ -8397,7 +8397,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A86">
         <v>85</v>
       </c>
@@ -8414,7 +8414,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A87">
         <v>86</v>
       </c>
@@ -8431,7 +8431,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A88">
         <v>87</v>
       </c>
@@ -8448,7 +8448,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A89">
         <v>88</v>
       </c>
@@ -8465,7 +8465,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A90">
         <v>89</v>
       </c>
@@ -8482,7 +8482,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A91">
         <v>90</v>
       </c>
@@ -8499,7 +8499,7 @@
         <v>0.45</v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A92">
         <v>91</v>
       </c>
@@ -8516,7 +8516,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A93">
         <v>92</v>
       </c>
@@ -8533,7 +8533,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A94">
         <v>93</v>
       </c>
@@ -8550,7 +8550,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A95">
         <v>94</v>
       </c>
@@ -8567,7 +8567,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A96">
         <v>95</v>
       </c>
@@ -8584,7 +8584,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A97">
         <v>96</v>
       </c>
@@ -8601,7 +8601,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A98">
         <v>97</v>
       </c>
@@ -8618,7 +8618,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A99">
         <v>98</v>
       </c>
@@ -8635,7 +8635,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A100">
         <v>99</v>
       </c>
@@ -8652,7 +8652,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.7">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A101">
         <v>100</v>
       </c>
@@ -8681,14 +8681,14 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED9894AF-30A9-4679-8E69-895319B0949F}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultRowHeight="17.649999999999999" x14ac:dyDescent="0.7"/>
+  <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="16.625" customWidth="1"/>
-    <col min="2" max="2" width="14.375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.59765625" customWidth="1"/>
+    <col min="2" max="2" width="14.3984375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.7">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>34</v>
       </c>
@@ -8699,7 +8699,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.7">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>17</v>
       </c>
@@ -8710,7 +8710,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.7">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>140</v>
       </c>
@@ -8721,7 +8721,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.7">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>155</v>
       </c>
@@ -8732,7 +8732,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.7">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>156</v>
       </c>
@@ -8743,7 +8743,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.7">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>157</v>
       </c>
@@ -8754,7 +8754,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.7">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>161</v>
       </c>
@@ -8765,7 +8765,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.7">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>37</v>
       </c>
@@ -8776,7 +8776,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.7">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>89</v>
       </c>
@@ -8787,7 +8787,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.7">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>90</v>
       </c>
@@ -8798,7 +8798,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.7">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>123</v>
       </c>
@@ -8809,7 +8809,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.7">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>124</v>
       </c>
@@ -8820,7 +8820,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.7">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
         <v>162</v>
       </c>
@@ -8831,7 +8831,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.7">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
         <v>217</v>
       </c>
@@ -8854,15 +8854,15 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F8655EA-A40E-4922-BEBE-C6CE0494F654}">
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultRowHeight="17.649999999999999" x14ac:dyDescent="0.7"/>
+  <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="16.625" customWidth="1"/>
-    <col min="2" max="2" width="11.625" customWidth="1"/>
-    <col min="3" max="3" width="16.375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.1875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.59765625" customWidth="1"/>
+    <col min="2" max="2" width="11.59765625" customWidth="1"/>
+    <col min="3" max="3" width="16.3984375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.19921875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.7">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>34</v>
       </c>
@@ -8888,17 +8888,17 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3DC603D6-2C96-4006-AE42-9221D8B477BE}">
   <dimension ref="A1:H21"/>
-  <sheetFormatPr defaultRowHeight="17.649999999999999" x14ac:dyDescent="0.7"/>
+  <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="17.125" customWidth="1"/>
-    <col min="2" max="2" width="8.1875" customWidth="1"/>
-    <col min="3" max="3" width="16.625" customWidth="1"/>
-    <col min="4" max="4" width="10.375" customWidth="1"/>
-    <col min="5" max="5" width="10.625" customWidth="1"/>
-    <col min="6" max="6" width="18.875" customWidth="1"/>
+    <col min="1" max="1" width="17.09765625" customWidth="1"/>
+    <col min="2" max="2" width="8.19921875" customWidth="1"/>
+    <col min="3" max="3" width="16.59765625" customWidth="1"/>
+    <col min="4" max="4" width="10.3984375" customWidth="1"/>
+    <col min="5" max="5" width="10.59765625" customWidth="1"/>
+    <col min="6" max="6" width="18.8984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.7">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -8924,7 +8924,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.7">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>118</v>
       </c>
@@ -8950,7 +8950,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.7">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>119</v>
       </c>
@@ -8976,7 +8976,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.7">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>120</v>
       </c>
@@ -9002,7 +9002,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.7">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>141</v>
       </c>
@@ -9028,7 +9028,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.7">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>142</v>
       </c>
@@ -9054,7 +9054,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.7">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>142</v>
       </c>
@@ -9080,7 +9080,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.7">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>182</v>
       </c>
@@ -9106,7 +9106,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.7">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>183</v>
       </c>
@@ -9132,7 +9132,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.7">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>184</v>
       </c>
@@ -9158,7 +9158,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.7">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>185</v>
       </c>
@@ -9184,7 +9184,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.7">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>186</v>
       </c>
@@ -9210,7 +9210,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.7">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
         <v>187</v>
       </c>
@@ -9236,7 +9236,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.7">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
         <v>218</v>
       </c>
@@ -9262,7 +9262,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.7">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
         <v>180</v>
       </c>
@@ -9285,7 +9285,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.7">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
         <v>181</v>
       </c>
@@ -9308,7 +9308,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.7">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
         <v>112</v>
       </c>
@@ -9331,7 +9331,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.7">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
         <v>113</v>
       </c>
@@ -9354,7 +9354,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.7">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
         <v>125</v>
       </c>
@@ -9377,7 +9377,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.7">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
         <v>126</v>
       </c>
@@ -9400,7 +9400,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.7">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
         <v>179</v>
       </c>
@@ -9435,16 +9435,16 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3FB3B4E8-C5C7-487A-BB3C-0105F4AA5D23}">
   <dimension ref="A1:F21"/>
-  <sheetFormatPr defaultRowHeight="17.649999999999999" x14ac:dyDescent="0.7"/>
+  <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="20.375" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="24.1875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="24.1875" customWidth="1"/>
-    <col min="5" max="5" width="13.875" customWidth="1"/>
-    <col min="6" max="6" width="15.625" customWidth="1"/>
+    <col min="1" max="1" width="20.3984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="24.19921875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="24.19921875" customWidth="1"/>
+    <col min="5" max="5" width="13.8984375" customWidth="1"/>
+    <col min="6" max="6" width="15.59765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.7">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -9464,7 +9464,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.7">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>98</v>
       </c>
@@ -9481,7 +9481,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.7">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>99</v>
       </c>
@@ -9501,7 +9501,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.7">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>100</v>
       </c>
@@ -9521,7 +9521,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.7">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>145</v>
       </c>
@@ -9541,7 +9541,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.7">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>148</v>
       </c>
@@ -9561,7 +9561,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.7">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>151</v>
       </c>
@@ -9581,7 +9581,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.7">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>210</v>
       </c>
@@ -9601,7 +9601,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.7">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>211</v>
       </c>
@@ -9621,7 +9621,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.7">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>212</v>
       </c>
@@ -9641,7 +9641,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.7">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>213</v>
       </c>
@@ -9661,7 +9661,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.7">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>214</v>
       </c>
@@ -9681,7 +9681,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.7">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
         <v>44</v>
       </c>
@@ -9701,7 +9701,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.7">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
         <v>101</v>
       </c>
@@ -9721,7 +9721,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.7">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
         <v>44</v>
       </c>
@@ -9741,7 +9741,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.7">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
         <v>101</v>
       </c>
@@ -9761,7 +9761,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.7">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
         <v>101</v>
       </c>
@@ -9781,7 +9781,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.7">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
         <v>44</v>
       </c>
@@ -9801,7 +9801,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.7">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.45">
       <c r="E21" s="2"/>
     </row>
   </sheetData>
@@ -9816,13 +9816,13 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CEE8DF46-D209-4D20-A42D-5A124B098697}">
   <dimension ref="A1:B9"/>
-  <sheetFormatPr defaultRowHeight="17.649999999999999" x14ac:dyDescent="0.7"/>
+  <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="16.625" customWidth="1"/>
-    <col min="2" max="2" width="11.125" customWidth="1"/>
+    <col min="1" max="1" width="16.59765625" customWidth="1"/>
+    <col min="2" max="2" width="11.09765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.7">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>34</v>
       </c>
@@ -9830,7 +9830,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.7">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>37</v>
       </c>
@@ -9838,7 +9838,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.7">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>17</v>
       </c>
@@ -9846,7 +9846,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.7">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>18</v>
       </c>
@@ -9854,7 +9854,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.7">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>19</v>
       </c>
@@ -9862,7 +9862,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.7">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>20</v>
       </c>
@@ -9870,7 +9870,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.7">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>21</v>
       </c>
@@ -9878,7 +9878,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.7">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>22</v>
       </c>
@@ -9886,7 +9886,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.7">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A9" s="3"/>
       <c r="B9" s="3"/>
     </row>

</xml_diff>